<commit_message>
chore: version 2.0.0 baseline push to GitHub
</commit_message>
<xml_diff>
--- a/009 变更记录/V003_to_V004_变更对比清单.xlsx
+++ b/009 变更记录/V003_to_V004_变更对比清单.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\长征文化\009 变更记录\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5BC6E04-660D-43E2-8CBC-88F7DD9CB813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0DBCC0B-E032-43C6-BE7B-8DDA5DEAE353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -276,10 +276,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>5步翻页：图片固定。时间→战役→会议→事件→意义 遗址/诗词/故事/人物/星火放 滚动页</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>每个节点信息面板最上面放高清照片
 （V003 修改日志 9.1.2 已记录）</t>
     <phoneticPr fontId="6" type="noConversion"/>
@@ -302,6 +298,10 @@
   </si>
   <si>
     <t>支持按关键字搜索节点</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>5步翻页：图片固定。时间→战役→会议→事件→意义 遗址/诗词/故事/人物/星火上传 滚动页</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -474,10 +474,31 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -489,27 +510,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,19 +827,19 @@
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
     </row>
     <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -857,18 +857,18 @@
       <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
     </row>
     <row r="5" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -886,7 +886,7 @@
       <c r="E5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="9" t="s">
         <v>60</v>
       </c>
     </row>
@@ -923,7 +923,7 @@
       <c r="E7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="9" t="s">
         <v>61</v>
       </c>
     </row>
@@ -943,7 +943,7 @@
       <c r="E8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="9" t="s">
         <v>64</v>
       </c>
     </row>
@@ -963,18 +963,18 @@
       <c r="E9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="10" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
     </row>
     <row r="11" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
@@ -992,7 +992,7 @@
       <c r="E11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="10" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       <c r="E12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="10" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       <c r="E13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="10" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       <c r="E14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="10" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       <c r="E15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="10" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       <c r="E16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="10" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
       <c r="E17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="10" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       <c r="E18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="10" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1157,13 +1157,13 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
     </row>
     <row r="21" spans="1:6" ht="82.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
@@ -1181,8 +1181,8 @@
       <c r="E21" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F21" s="18" t="s">
-        <v>76</v>
+      <c r="F21" s="11" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1193,7 +1193,7 @@
         <v>45</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>46</v>
@@ -1201,8 +1201,8 @@
       <c r="E22" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="18" t="s">
-        <v>77</v>
+      <c r="F22" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1213,7 +1213,7 @@
         <v>48</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>49</v>
@@ -1221,8 +1221,8 @@
       <c r="E23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F23" s="19" t="s">
-        <v>78</v>
+      <c r="F23" s="12" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>51</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>52</v>
@@ -1241,8 +1241,8 @@
       <c r="E24" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F24" s="19" t="s">
-        <v>79</v>
+      <c r="F24" s="12" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1253,7 +1253,7 @@
         <v>53</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>54</v>
@@ -1261,8 +1261,8 @@
       <c r="E25" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F25" s="19" t="s">
-        <v>80</v>
+      <c r="F25" s="12" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1273,7 +1273,7 @@
         <v>55</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>56</v>
@@ -1281,8 +1281,8 @@
       <c r="E26" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="20" t="s">
-        <v>81</v>
+      <c r="F26" s="13" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="52.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1293,7 +1293,7 @@
         <v>57</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>58</v>
@@ -1301,18 +1301,18 @@
       <c r="E27" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F27" s="20" t="s">
-        <v>82</v>
+      <c r="F27" s="13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>